<commit_message>
Split mark list into per-subject sheets styled like reference
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BzKKfTW8peYFM8N3VFGV68
</commit_message>
<xml_diff>
--- a/11th_Std_Mark_List.xlsx
+++ b/11th_Std_Mark_List.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mark List" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Physics" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemistry" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maths" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,16 +28,21 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <color rgb="00FF0000"/>
+      <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00FF0000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00002060"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -44,17 +51,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002E75B6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
+        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -67,42 +64,26 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="009BC2E6"/>
-      </left>
-      <right style="thin">
-        <color rgb="009BC2E6"/>
-      </right>
-      <top style="thin">
-        <color rgb="009BC2E6"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="009BC2E6"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -469,52 +450,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>11TH STD MARK LIST</t>
-        </is>
-      </c>
+          <t>11TH STD PHYSICS  MARK LIST</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>NAMES</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>PHYSICS (30)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>CHEMISTRY (25)</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>MATHS (30)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>TOTAL (85)</t>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>OUT OF 30</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Chaitanya</t>
         </is>
@@ -522,180 +486,352 @@
       <c r="B3" s="4" t="n">
         <v>16.5</v>
       </c>
-      <c r="C3" s="4" t="n">
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Teja Shree</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Harish</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Pranesh</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Yashwanth</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Karthikeyan</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Tharangini</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Manoranjan</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Srinidhini</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>11TH STD CHEMISTRY  MARK LIST</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>NAMES</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>OUT OF 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Chaitanya</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="D3" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="E3" s="4">
-        <f>SUM(B3:D3)</f>
-        <v/>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Karthikeyan</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="C4" s="6" t="n">
+      <c r="B4" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="D4" s="6" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="E4" s="6">
-        <f>SUM(B4:D4)</f>
-        <v/>
-      </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Teja Shree</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Pranesh</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="C5" s="4" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="D5" s="4" t="n">
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Manoranjan</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
         <v>11.5</v>
       </c>
-      <c r="E5" s="4">
-        <f>SUM(B5:D5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Pranesh</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="E6" s="6">
-        <f>SUM(B6:D6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tharangini</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Harish</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="E7" s="4">
-        <f>SUM(B7:D7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Tharangini</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="E8" s="6">
-        <f>SUM(B8:D8)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Manoranjan</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
         <v>8.5</v>
       </c>
-      <c r="C9" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="E9" s="4">
-        <f>SUM(B9:D9)</f>
-        <v/>
-      </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Srinidhini</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="4" t="n">
         <v>8.5</v>
       </c>
-      <c r="C10" s="6" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="E10" s="6">
-        <f>SUM(B10:D10)</f>
-        <v/>
-      </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Yashwanth</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="C11" s="4" t="n">
         <v>5.5</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="E11" s="4">
-        <f>SUM(B11:D11)</f>
-        <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>11TH STD MATHS  MARK LIST</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>NAMES</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>OUT OF 30</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Chaitanya</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Harish</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Karthikeyan</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Pranesh</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Teja Shree</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tharangini</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>11.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Manoranjan</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Srinidhini</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Yashwanth</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>7.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Put subject tables side by side on one sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BzKKfTW8peYFM8N3VFGV68
</commit_message>
<xml_diff>
--- a/11th_Std_Mark_List.xlsx
+++ b/11th_Std_Mark_List.xlsx
@@ -7,9 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Physics" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chemistry" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maths" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mark List" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +26,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FF0000"/>
       <sz val="12"/>
@@ -448,13 +445,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -464,6 +467,18 @@
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>11TH STD CHEMISTRY  MARK LIST</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="n"/>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>11TH STD MATHS  MARK LIST</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -476,6 +491,26 @@
           <t>OUT OF 30</t>
         </is>
       </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>NAMES</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>OUT OF 25</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>NAMES</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>OUT OF 30</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -486,6 +521,22 @@
       <c r="B3" s="4" t="n">
         <v>16.5</v>
       </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Chaitanya</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Chaitanya</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -496,6 +547,22 @@
       <c r="B4" s="4" t="n">
         <v>13</v>
       </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Karthikeyan</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Harish</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -506,6 +573,22 @@
       <c r="B5" s="4" t="n">
         <v>12</v>
       </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Teja Shree</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Karthikeyan</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>12.5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -516,6 +599,22 @@
       <c r="B6" s="4" t="n">
         <v>11.5</v>
       </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Pranesh</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>Pranesh</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>12.5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -526,6 +625,22 @@
       <c r="B7" s="4" t="n">
         <v>11.5</v>
       </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Manoranjan</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Teja Shree</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>11.5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -536,6 +651,22 @@
       <c r="B8" s="4" t="n">
         <v>11</v>
       </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Tharangini</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Tharangini</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>11.5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -546,6 +677,22 @@
       <c r="B9" s="4" t="n">
         <v>10.5</v>
       </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Harish</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>Manoranjan</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -556,6 +703,22 @@
       <c r="B10" s="4" t="n">
         <v>8.5</v>
       </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Srinidhini</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Srinidhini</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>8.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -566,273 +729,30 @@
       <c r="B11" s="4" t="n">
         <v>8.5</v>
       </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Yashwanth</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>Yashwanth</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>7.5</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>11TH STD CHEMISTRY  MARK LIST</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>NAMES</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>OUT OF 25</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Chaitanya</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Karthikeyan</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Teja Shree</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>13.5</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Pranesh</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Manoranjan</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>11.5</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Tharangini</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Harish</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>8.5</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Srinidhini</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>8.5</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Yashwanth</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="n">
-        <v>5.5</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>11TH STD MATHS  MARK LIST</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>NAMES</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>OUT OF 30</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Chaitanya</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Harish</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Karthikeyan</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>12.5</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Pranesh</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>12.5</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Teja Shree</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>11.5</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Tharangini</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>11.5</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Manoranjan</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Srinidhini</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>8.5</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Yashwanth</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="n">
-        <v>7.5</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Maths marks to 24/10 test
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BzKKfTW8peYFM8N3VFGV68
</commit_message>
<xml_diff>
--- a/11th_Std_Mark_List.xlsx
+++ b/11th_Std_Mark_List.xlsx
@@ -52,7 +52,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -66,11 +66,32 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -82,6 +103,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -466,19 +488,19 @@
           <t>11TH STD PHYSICS  MARK LIST</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
+      <c r="B1" s="5" t="n"/>
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>11TH STD CHEMISTRY  MARK LIST</t>
         </is>
       </c>
-      <c r="E1" s="2" t="n"/>
+      <c r="E1" s="5" t="n"/>
       <c r="G1" s="1" t="inlineStr">
         <is>
           <t>11TH STD MATHS  MARK LIST</t>
         </is>
       </c>
-      <c r="H1" s="2" t="n"/>
+      <c r="H1" s="5" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -535,7 +557,7 @@
         </is>
       </c>
       <c r="H3" s="4" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -557,11 +579,11 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Harish</t>
+          <t>Teja Shree</t>
         </is>
       </c>
       <c r="H4" s="4" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
@@ -583,11 +605,11 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Karthikeyan</t>
+          <t>Pranesh</t>
         </is>
       </c>
       <c r="H5" s="4" t="n">
-        <v>12.5</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="6">
@@ -609,11 +631,11 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Pranesh</t>
+          <t>Yashwanth</t>
         </is>
       </c>
       <c r="H6" s="4" t="n">
-        <v>12.5</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="7">
@@ -635,11 +657,11 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Teja Shree</t>
+          <t>Harish</t>
         </is>
       </c>
       <c r="H7" s="4" t="n">
-        <v>11.5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -661,11 +683,11 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Tharangini</t>
+          <t>Karthikeyan</t>
         </is>
       </c>
       <c r="H8" s="4" t="n">
-        <v>11.5</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="9">
@@ -687,11 +709,11 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Manoranjan</t>
+          <t>Tharangini</t>
         </is>
       </c>
       <c r="H9" s="4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10">
@@ -713,11 +735,11 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Srinidhini</t>
+          <t>Manoranjan</t>
         </is>
       </c>
       <c r="H10" s="4" t="n">
-        <v>8.5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11">
@@ -739,7 +761,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Yashwanth</t>
+          <t>Srinidhini</t>
         </is>
       </c>
       <c r="H11" s="4" t="n">

</xml_diff>